<commit_message>
Labs: open workbooks locally, not via OneDrive; Lab 6 skill fixes
- Shared setup step: copy the lab workbook into a local work-c34 folder and
  open it in desktop Excel; no onedrive.com upload or Excel for the web.
  OneDrive is kept only for custom skills (Labs 6, 8) and attaching files.
- Lab 6: Custom skills switch + "Add in OneDrive" button, Refresh wait,
  check the right workbook is open, troubleshooting for a missing
  tblInterviews. Workbook now opens on the Interviews sheet.
- About_This_Data: taller rows for long wrapped meanings.
- Lab 5 skill-folder wording (from the earlier pending edit).
- Rebuilt lab PDFs, sample prompts, prompts page, LG/LP/deck.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-05-built-in-skills-visual-and-finance/data/BrightPath_HR_Outsourcing_Finance.xlsx
+++ b/labs/lab-05-built-in-skills-visual-and-finance/data/BrightPath_HR_Outsourcing_Finance.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>tblClientMonths</t>
@@ -570,7 +570,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>tblClients</t>
@@ -604,7 +604,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>Headcount_Budget</t>
@@ -621,7 +621,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>Definitions</t>

</xml_diff>